<commit_message>
Refresh final DraftOps data and live tooling
</commit_message>
<xml_diff>
--- a/数据/上传此文件即可（选秀+里程碑问题选手答题卡_完整下拉选项已填）.xlsx
+++ b/数据/上传此文件即可（选秀+里程碑问题选手答题卡_完整下拉选项已填）.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" state="visible" r:id="rId1"/>
@@ -165,15 +165,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,100 +543,100 @@
   <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="4" customWidth="1" style="12" min="1" max="1"/>
-    <col width="100" customWidth="1" style="12" min="2" max="2"/>
+    <col width="4" customWidth="1" style="11" min="1" max="1"/>
+    <col width="100" customWidth="1" style="11" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" s="12">
-      <c r="A1" s="13" t="inlineStr">
+    <row r="1" ht="36" customHeight="1" s="11">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Draftcode 24 · 选手答题卡（提交模板）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1" s="12">
+    <row r="2" ht="17" customHeight="1" s="11">
       <c r="B2" s="8" t="n"/>
     </row>
-    <row r="3" ht="17" customHeight="1" s="12">
+    <row r="3" ht="17" customHeight="1" s="11">
       <c r="B3" s="9" t="inlineStr">
         <is>
           <t>一、本文件共 4 张表，请按顺序填写：</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1" s="12">
+    <row r="4" ht="34" customHeight="1" s="11">
       <c r="B4" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    ①「队伍信息」——务必填写 队伍ID（team_id），这是计分系统识别你队伍的唯一依据，不可留空、不可改格式。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1" s="12">
+    <row r="5" ht="17" customHeight="1" s="11">
       <c r="B5" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    ②「选秀名单预测」——对首轮 1–30 顺位逐个预测被选中的球员（每队 2.4 分，共 72 分）。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="17" customHeight="1" s="12">
+    <row r="6" ht="17" customHeight="1" s="11">
       <c r="B6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    ③「里程碑预测」——回答 7 道里程碑问题（每题 4 分，共 28 分）。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="17" customHeight="1" s="12">
+    <row r="7" ht="17" customHeight="1" s="11">
       <c r="B7" s="8" t="n"/>
     </row>
-    <row r="8" ht="17" customHeight="1" s="12">
+    <row r="8" ht="17" customHeight="1" s="11">
       <c r="B8" s="9" t="inlineStr">
         <is>
           <t>二、填写规则：</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1" s="12">
+    <row r="9" ht="34" customHeight="1" s="11">
       <c r="B9" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    1. 选秀名单预测的“预测球员”一栏，请务必从单元格下拉列表中选择，不要手动输入（手输无法被识别计分）。</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="17" customHeight="1" s="12">
+    <row r="10" ht="17" customHeight="1" s="11">
       <c r="B10" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    2. 里程碑数字题请只填数字；Q6 请从下拉选择机构名。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="17" customHeight="1" s="12">
+    <row r="11" ht="17" customHeight="1" s="11">
       <c r="B11" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    3. 黄色底色单元格为需要你填写的内容；请勿增删行、列或修改表头。</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="17" customHeight="1" s="12">
+    <row r="12" ht="17" customHeight="1" s="11">
       <c r="B12" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">    4. 一个文件代表一支队伍。提交后系统按截止时间锁定，不可修改。</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="17" customHeight="1" s="12">
+    <row r="13" ht="17" customHeight="1" s="11">
       <c r="B13" s="8" t="n"/>
     </row>
-    <row r="14" ht="34" customHeight="1" s="12">
+    <row r="14" ht="34" customHeight="1" s="11">
       <c r="B14" s="9" t="inlineStr">
         <is>
           <t>三、计分口径：总分 = 代码评分×30% + 路演×30% + (选秀名单+里程碑)×40%。详见《需求冻结_设计基准》。</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="17" customHeight="1" s="12">
+    <row r="15" ht="17" customHeight="1" s="11">
       <c r="B15" s="8" t="n"/>
     </row>
-    <row r="16" ht="17" customHeight="1" s="12">
+    <row r="16" ht="17" customHeight="1" s="11">
       <c r="B16" s="9" t="inlineStr">
         <is>
           <t>四、提交方式与截止时间：6/24 8：00</t>
@@ -660,55 +660,55 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="26.6328125" customWidth="1" style="12" min="1" max="1"/>
-    <col width="40" customWidth="1" style="12" min="2" max="2"/>
+    <col width="26.6328125" customWidth="1" style="11" min="1" max="1"/>
+    <col width="40" customWidth="1" style="11" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="12">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>队伍信息</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1" s="12">
+    <row r="2" ht="17" customHeight="1" s="11">
       <c r="A2" s="6" t="inlineStr">
         <is>
           <t>队伍ID</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="13" t="inlineStr">
         <is>
           <t>Team21</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="17" customHeight="1" s="12">
+    <row r="3" ht="17" customHeight="1" s="11">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>队伍名称</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>启元开物</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="17" customHeight="1" s="12">
+    <row r="4" ht="17" customHeight="1" s="11">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>队长姓名 / 联系方式</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>肖云涵/13508349471</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1" s="12"/>
-    <row r="6" ht="34" customHeight="1" s="12">
+    <row r="5" ht="34" customHeight="1" s="11"/>
+    <row r="6" ht="34" customHeight="1" s="11">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>提示：team_id 由组委会分配，格式为 Team01–Team27（如 Team01），请勿自行更改。</t>
@@ -732,34 +732,34 @@
   <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="5.36328125" customWidth="1" style="12" min="1" max="1"/>
-    <col width="22" customWidth="1" style="12" min="2" max="2"/>
-    <col width="22" customWidth="1" style="12" min="4" max="4"/>
-    <col width="10.26953125" customWidth="1" style="12" min="5" max="5"/>
+    <col width="5.36328125" customWidth="1" style="11" min="1" max="1"/>
+    <col width="22" customWidth="1" style="11" min="2" max="2"/>
+    <col width="22" customWidth="1" style="11" min="4" max="4"/>
+    <col width="10.26953125" customWidth="1" style="11" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="12">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="34" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>姓名</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="10" t="inlineStr">
         <is>
           <t>位置</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="10" t="inlineStr">
         <is>
           <t>学校/俱乐部</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="10" t="inlineStr">
         <is>
           <t>国家/地区</t>
         </is>
@@ -3879,19 +3879,19 @@
   <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="8" customWidth="1" style="12" min="1" max="1"/>
-    <col width="28" customWidth="1" style="12" min="2" max="2"/>
-    <col width="53.81640625" customWidth="1" style="12" min="3" max="3"/>
+    <col width="8" customWidth="1" style="11" min="1" max="1"/>
+    <col width="28" customWidth="1" style="11" min="2" max="2"/>
+    <col width="53.81640625" customWidth="1" style="11" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="12">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>二、选秀名单预测　|　首轮 1–30 顺位逐队预测　|　每队命中 2.4 分（满分 72）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1" s="12">
+    <row r="2" ht="17" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>顺位</t>
@@ -3908,7 +3908,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="17" customHeight="1" s="12">
+    <row r="3" ht="17" customHeight="1" s="11">
       <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="17" customHeight="1" s="12">
+    <row r="4" ht="17" customHeight="1" s="11">
       <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
@@ -3938,7 +3938,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1" s="12">
+    <row r="5" ht="17" customHeight="1" s="11">
       <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
@@ -3953,7 +3953,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="17" customHeight="1" s="12">
+    <row r="6" ht="17" customHeight="1" s="11">
       <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
@@ -3968,7 +3968,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17" customHeight="1" s="12">
+    <row r="7" ht="17" customHeight="1" s="11">
       <c r="A7" s="3" t="n">
         <v>5</v>
       </c>
@@ -3983,7 +3983,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="17" customHeight="1" s="12">
+    <row r="8" ht="17" customHeight="1" s="11">
       <c r="A8" s="3" t="n">
         <v>6</v>
       </c>
@@ -3994,11 +3994,11 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>达柳斯 阿卡夫</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="17" customHeight="1" s="12">
+          <t>金斯顿 弗莱明斯</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1" s="11">
       <c r="A9" s="3" t="n">
         <v>7</v>
       </c>
@@ -4009,11 +4009,11 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>迈克尔 布朗</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="17" customHeight="1" s="12">
+          <t>达柳斯 阿卡夫</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1" s="11">
       <c r="A10" s="3" t="n">
         <v>8</v>
       </c>
@@ -4024,11 +4024,11 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>阿达伊 马拉</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="17" customHeight="1" s="12">
+          <t>纳撒尼尔 阿门特</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1" s="11">
       <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
@@ -4043,7 +4043,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="17" customHeight="1" s="12">
+    <row r="12" ht="17" customHeight="1" s="11">
       <c r="A12" s="3" t="n">
         <v>10</v>
       </c>
@@ -4054,11 +4054,11 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>金斯顿 弗莱明斯</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1" s="12">
+          <t>卡里姆 洛佩兹</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1" s="11">
       <c r="A13" s="3" t="n">
         <v>11</v>
       </c>
@@ -4069,11 +4069,11 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>纳撒尼尔 阿门特</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1" s="12">
+          <t>小拉巴伦 菲隆</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1" s="11">
       <c r="A14" s="3" t="n">
         <v>12</v>
       </c>
@@ -4084,11 +4084,11 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>亚克塞尔 伦德伯格</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1" s="12">
+          <t>阿达伊 马拉</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1" s="11">
       <c r="A15" s="3" t="n">
         <v>13</v>
       </c>
@@ -4099,11 +4099,11 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>卡里姆 洛佩兹</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1" s="12">
+          <t>亚克塞尔 伦德伯格</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1" s="11">
       <c r="A16" s="3" t="n">
         <v>14</v>
       </c>
@@ -4114,11 +4114,11 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>小莫雷兹 约翰逊</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="17" customHeight="1" s="12">
+          <t>阿伦 格雷夫斯</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1" s="11">
       <c r="A17" s="3" t="n">
         <v>15</v>
       </c>
@@ -4129,11 +4129,11 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>阿伦 格雷夫斯</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="17" customHeight="1" s="12">
+          <t>卡梅隆 卡尔</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1" s="11">
       <c r="A18" s="3" t="n">
         <v>16</v>
       </c>
@@ -4144,11 +4144,11 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>汉内斯 施泰因巴赫</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="17" customHeight="1" s="12">
+          <t>戴林 斯温</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1" s="11">
       <c r="A19" s="3" t="n">
         <v>17</v>
       </c>
@@ -4159,11 +4159,11 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>克里斯 塞纳克</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1" s="12">
+          <t>小莫雷兹 约翰逊</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1" s="11">
       <c r="A20" s="3" t="n">
         <v>18</v>
       </c>
@@ -4178,7 +4178,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1" s="12">
+    <row r="21" ht="17" customHeight="1" s="11">
       <c r="A21" s="3" t="n">
         <v>19</v>
       </c>
@@ -4189,11 +4189,11 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>小拉巴伦 菲隆</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="17" customHeight="1" s="12">
+          <t>迈克尔 布朗</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1" s="11">
       <c r="A22" s="3" t="n">
         <v>20</v>
       </c>
@@ -4208,7 +4208,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="17" customHeight="1" s="12">
+    <row r="23" ht="17" customHeight="1" s="11">
       <c r="A23" s="3" t="n">
         <v>21</v>
       </c>
@@ -4219,11 +4219,11 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>卡梅隆 卡尔</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="17" customHeight="1" s="12">
+          <t>以赛亚 埃文斯</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1" s="11">
       <c r="A24" s="3" t="n">
         <v>22</v>
       </c>
@@ -4234,11 +4234,11 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>戴林 斯温</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="17" customHeight="1" s="12">
+          <t>汉内斯 施泰因巴赫</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1" s="11">
       <c r="A25" s="3" t="n">
         <v>23</v>
       </c>
@@ -4249,11 +4249,11 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>埃布卡 奥科里</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17" customHeight="1" s="12">
+          <t>塞尔吉奥 德拉雷亚</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1" s="11">
       <c r="A26" s="3" t="n">
         <v>24</v>
       </c>
@@ -4264,11 +4264,11 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>以赛亚 埃文斯</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="17" customHeight="1" s="12">
+          <t>埃布卡 奥科里</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1" s="11">
       <c r="A27" s="3" t="n">
         <v>25</v>
       </c>
@@ -4283,7 +4283,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="17" customHeight="1" s="12">
+    <row r="28" ht="17" customHeight="1" s="11">
       <c r="A28" s="3" t="n">
         <v>26</v>
       </c>
@@ -4294,11 +4294,11 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>小塔里斯 里德</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="17" customHeight="1" s="12">
+          <t>亨利 维萨尔</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1" s="11">
       <c r="A29" s="3" t="n">
         <v>27</v>
       </c>
@@ -4309,11 +4309,11 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>塞尔吉奥 德拉雷亚</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="17" customHeight="1" s="12">
+          <t>克里斯 塞纳克</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="17" customHeight="1" s="11">
       <c r="A30" s="3" t="n">
         <v>28</v>
       </c>
@@ -4328,7 +4328,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="17" customHeight="1" s="12">
+    <row r="31" ht="17" customHeight="1" s="11">
       <c r="A31" s="3" t="n">
         <v>29</v>
       </c>
@@ -4339,11 +4339,11 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>亨利 维萨尔</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="17" customHeight="1" s="12">
+          <t>小塔里斯 里德</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="17" customHeight="1" s="11">
       <c r="A32" s="3" t="n">
         <v>30</v>
       </c>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>杰克 卡伊尔</t>
+          <t>泰勒 比洛多</t>
         </is>
       </c>
     </row>
@@ -4380,20 +4380,20 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col width="8" customWidth="1" style="12" min="1" max="1"/>
-    <col width="16" customWidth="1" style="12" min="2" max="2"/>
-    <col width="56" customWidth="1" style="12" min="3" max="3"/>
-    <col width="22" customWidth="1" style="12" min="4" max="6"/>
+    <col width="8" customWidth="1" style="11" min="1" max="1"/>
+    <col width="16" customWidth="1" style="11" min="2" max="2"/>
+    <col width="56" customWidth="1" style="11" min="3" max="3"/>
+    <col width="22" customWidth="1" style="11" min="4" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="12">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="11">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>三、里程碑事件预测　|　共 7 题　|　每题命中 4 分（满分 28）</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1" s="12">
+    <row r="2" ht="17" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>题号</t>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="46" customHeight="1" s="12">
+    <row r="3" ht="46" customHeight="1" s="11">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Q1</t>
@@ -4452,10 +4452,10 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" ht="46" customHeight="1" s="12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1" s="11">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Q2</t>
@@ -4485,7 +4485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" ht="46" customHeight="1" s="12">
+    <row r="5" ht="46" customHeight="1" s="11">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Q3</t>
@@ -4515,7 +4515,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" ht="46" customHeight="1" s="12">
+    <row r="6" ht="46" customHeight="1" s="11">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Q4</t>
@@ -4542,10 +4542,10 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" ht="46" customHeight="1" s="12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1" s="11">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Q5</t>
@@ -4575,7 +4575,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" ht="46" customHeight="1" s="12">
+    <row r="8" ht="46" customHeight="1" s="11">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Q6</t>
@@ -4607,7 +4607,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="46" customHeight="1" s="12">
+    <row r="9" ht="46" customHeight="1" s="11">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Q7</t>

</xml_diff>